<commit_message>
Content: rubric system (useful / fun / sales), week-2 speaker-announcement drafts, plan rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015DfynR8ViCbDyQMuNVS5SH
</commit_message>
<xml_diff>
--- a/content/plan/kontent-plan-RESHENO.xlsx
+++ b/content/plan/kontent-plan-RESHENO.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Как пользоваться" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'План'!$A$3:$O$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'План'!$A$3:$O$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O30"/>
+  <dimension ref="A1:O38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2527,13 +2527,565 @@
       </c>
       <c r="O30" s="5" t="inlineStr"/>
     </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Пн 05.10 · Тизер «На этой неделе раскрываем всех спикеров»</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Пост + сторис</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K31" s="4">
+        <f>IF(COUNTIF(F31:J31,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F31:J31,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Готов</t>
+        </is>
+      </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/1-pn-05.10-tizer.md · Figma: «Неделя 2 — спикеры»</t>
+        </is>
+      </c>
+      <c r="N31" s="5" t="inlineStr"/>
+      <c r="O31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Вт 06.10 · Спикеры трека MONEY</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Пост + карусель</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K32" s="4">
+        <f>IF(COUNTIF(F32:J32,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F32:J32,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M32" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/2-vt-06.10-money.md · Figma</t>
+        </is>
+      </c>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t>Нужны имена, должности, темы, фото, ники; пригласить спикеров соавторами</t>
+        </is>
+      </c>
+      <c r="O32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Ср 07.10 · Спикеры трека CLIENT</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Пост + карусель</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K33" s="4">
+        <f>IF(COUNTIF(F33:J33,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F33:J33,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/3-sr-07.10-client.md · Figma</t>
+        </is>
+      </c>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>То же</t>
+        </is>
+      </c>
+      <c r="O33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Чт 08.10 · Спикеры трека TEAM</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Пост + карусель</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K34" s="4">
+        <f>IF(COUNTIF(F34:J34,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F34:J34,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/4-cht-08.10-team.md · Figma</t>
+        </is>
+      </c>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t>То же</t>
+        </is>
+      </c>
+      <c r="O34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Пт 09.10 · Спикеры треков GROWTH + FUTURE</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Пост + карусель</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K35" s="4">
+        <f>IF(COUNTIF(F35:J35,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F35:J35,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/5-pt-09.10-growth-future.md · Figma</t>
+        </is>
+      </c>
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t>То же</t>
+        </is>
+      </c>
+      <c r="O35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Сб 10.10 · «Все спикеры РЕШЕНО» — закрепить</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Пост + карусель</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K36" s="4">
+        <f>IF(COUNTIF(F36:J36,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F36:J36,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/6-sb-10.10-vse-spikery.md · Figma</t>
+        </is>
+      </c>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>Открепить манифест, закрепить этот пост</t>
+        </is>
+      </c>
+      <c r="O36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Вс 11.10 · Опрос «Чей разбор ждёте больше всего?»</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Опрос + сторис</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K37" s="4">
+        <f>IF(COUNTIF(F37:J37,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F37:J37,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/7-vs-11.10-opros.md · Figma</t>
+        </is>
+      </c>
+      <c r="N37" s="5" t="inlineStr"/>
+      <c r="O37" s="5" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Каждый день · Сторис-отсчёт «До форума N дней» + сторис каждого спикера</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Сторис</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Отсчёт</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K38" s="4">
+        <f>IF(COUNTIF(F38:J38,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F38:J38,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Готов</t>
+        </is>
+      </c>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/instagram/README.md · Figma</t>
+        </is>
+      </c>
+      <c r="N38" s="5" t="inlineStr">
+        <is>
+          <t>Вт 38, Ср 37, Чт 36, Пт 35, Сб 34, Вс 33</t>
+        </is>
+      </c>
+      <c r="O38" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:O30"/>
+  <autoFilter ref="A3:O38"/>
   <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F4:J80">
+  <conditionalFormatting sqref="F4:J88">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Выложено"</formula>
     </cfRule>
@@ -2544,26 +3096,26 @@
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K4:K80">
+  <conditionalFormatting sqref="K4:K88">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
       <formula>"Готово"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L80">
+  <conditionalFormatting sqref="L4:L88">
     <cfRule type="cellIs" priority="5" operator="notEqual" dxfId="3">
       <formula>"Готов"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:E30">
+  <conditionalFormatting sqref="A4:E38">
     <cfRule type="expression" priority="6" dxfId="4">
       <formula>$K4="Готово"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F4:J80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F4:J88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Нужно,Выложено,—"</formula1>
     </dataValidation>
-    <dataValidation sqref="L4:L80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L4:L88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Готов,Нужно снять,Нужно сделать,Ждём цифры опроса"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2628,11 +3180,11 @@
         </is>
       </c>
       <c r="B3" s="9">
-        <f>COUNTIF(План!F4:F80,"Нужно")+COUNTIF(План!F4:F80,"Выложено")</f>
+        <f>COUNTIF(План!F4:F88,"Нужно")+COUNTIF(План!F4:F88,"Выложено")</f>
         <v/>
       </c>
       <c r="C3" s="9">
-        <f>COUNTIF(План!F4:F80,"Выложено")</f>
+        <f>COUNTIF(План!F4:F88,"Выложено")</f>
         <v/>
       </c>
       <c r="D3" s="9">
@@ -2651,11 +3203,11 @@
         </is>
       </c>
       <c r="B4" s="9">
-        <f>COUNTIF(План!G4:G80,"Нужно")+COUNTIF(План!G4:G80,"Выложено")</f>
+        <f>COUNTIF(План!G4:G88,"Нужно")+COUNTIF(План!G4:G88,"Выложено")</f>
         <v/>
       </c>
       <c r="C4" s="9">
-        <f>COUNTIF(План!G4:G80,"Выложено")</f>
+        <f>COUNTIF(План!G4:G88,"Выложено")</f>
         <v/>
       </c>
       <c r="D4" s="9">
@@ -2674,11 +3226,11 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <f>COUNTIF(План!H4:H80,"Нужно")+COUNTIF(План!H4:H80,"Выложено")</f>
+        <f>COUNTIF(План!H4:H88,"Нужно")+COUNTIF(План!H4:H88,"Выложено")</f>
         <v/>
       </c>
       <c r="C5" s="9">
-        <f>COUNTIF(План!H4:H80,"Выложено")</f>
+        <f>COUNTIF(План!H4:H88,"Выложено")</f>
         <v/>
       </c>
       <c r="D5" s="9">
@@ -2697,11 +3249,11 @@
         </is>
       </c>
       <c r="B6" s="9">
-        <f>COUNTIF(План!I4:I80,"Нужно")+COUNTIF(План!I4:I80,"Выложено")</f>
+        <f>COUNTIF(План!I4:I88,"Нужно")+COUNTIF(План!I4:I88,"Выложено")</f>
         <v/>
       </c>
       <c r="C6" s="9">
-        <f>COUNTIF(План!I4:I80,"Выложено")</f>
+        <f>COUNTIF(План!I4:I88,"Выложено")</f>
         <v/>
       </c>
       <c r="D6" s="9">
@@ -2720,11 +3272,11 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>COUNTIF(План!J4:J80,"Нужно")+COUNTIF(План!J4:J80,"Выложено")</f>
+        <f>COUNTIF(План!J4:J88,"Нужно")+COUNTIF(План!J4:J88,"Выложено")</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>COUNTIF(План!J4:J80,"Выложено")</f>
+        <f>COUNTIF(План!J4:J88,"Выложено")</f>
         <v/>
       </c>
       <c r="D7" s="9">
@@ -2773,7 +3325,7 @@
         </is>
       </c>
       <c r="B10" s="13">
-        <f>COUNTA(План!C4:C80)</f>
+        <f>COUNTA(План!C4:C88)</f>
         <v/>
       </c>
       <c r="C10" s="13" t="n"/>
@@ -2787,7 +3339,7 @@
         </is>
       </c>
       <c r="B11" s="13">
-        <f>COUNTIF(План!K4:K80,"Готово")</f>
+        <f>COUNTIF(План!K4:K88,"Готово")</f>
         <v/>
       </c>
       <c r="C11" s="13" t="n"/>
@@ -2801,7 +3353,7 @@
         </is>
       </c>
       <c r="B12" s="13">
-        <f>COUNTIF(План!L4:L80,"&lt;&gt;Готов")-COUNTBLANK(План!L4:L80)</f>
+        <f>COUNTIF(План!L4:L88,"&lt;&gt;Готов")-COUNTBLANK(План!L4:L88)</f>
         <v/>
       </c>
       <c r="C12" s="13" t="n"/>

</xml_diff>

<commit_message>
Weeks 3–4 (12.10–25.10): 9 carousels, 5 memes, 14 countdown stories, texts for all platforms, checklist; plan rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015DfynR8ViCbDyQMuNVS5SH
</commit_message>
<xml_diff>
--- a/content/plan/kontent-plan-RESHENO.xlsx
+++ b/content/plan/kontent-plan-RESHENO.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Как пользоваться" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'План'!$A$3:$O$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'План'!$A$3:$O$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:O53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2533,22 +2533,22 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>9. Неделя 2 — спикеры</t>
+          <t>10. Недели 3–4</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Пн 05.10 · Тизер «На этой неделе раскрываем всех спикеров»</t>
+          <t>Пн 12.10 · Знакомьтесь: это зубр + сбор имени</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Пост + сторис</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Спикеры</t>
+          <t>Знакомство</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -2587,10 +2587,14 @@
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/1-pn-05.10-tizer.md · Figma: «Неделя 2 — спикеры»</t>
-        </is>
-      </c>
-      <c r="N31" s="5" t="inlineStr"/>
+          <t>content/nedeli-3-4_12.10-25.10/01-pn-12.10-znakomtes-zubr/</t>
+        </is>
+      </c>
+      <c r="N31" s="5" t="inlineStr">
+        <is>
+          <t>Решить про подарок автору имени</t>
+        </is>
+      </c>
       <c r="O31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
@@ -2599,22 +2603,22 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>9. Неделя 2 — спикеры</t>
+          <t>10. Недели 3–4</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Вт 06.10 · Спикеры трека MONEY</t>
+          <t>Вт 13.10 · Сколько стоит потерянный клиент + чек-лист</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Пост + карусель</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Спикеры</t>
+          <t>Польза</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -2648,17 +2652,17 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Ждём цифры опроса</t>
+          <t>Готов</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/2-vt-06.10-money.md · Figma</t>
+          <t>content/nedeli-3-4_12.10-25.10/02-vt-13.10-poteryannyy-klient/</t>
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>Нужны имена, должности, темы, фото, ники; пригласить спикеров соавторами</t>
+          <t>Сразу после поста — чек-лист в Telegram</t>
         </is>
       </c>
       <c r="O32" s="5" t="inlineStr"/>
@@ -2669,22 +2673,22 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>9. Неделя 2 — спикеры</t>
+          <t>10. Недели 3–4</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Ср 07.10 · Спикеры трека CLIENT</t>
+          <t>Ср 14.10 · Мем «Родительский чат в 23:47»</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Пост + карусель</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Спикеры</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2718,19 +2722,15 @@
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>Ждём цифры опроса</t>
+          <t>Готов</t>
         </is>
       </c>
       <c r="M33" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/3-sr-07.10-client.md · Figma</t>
-        </is>
-      </c>
-      <c r="N33" s="5" t="inlineStr">
-        <is>
-          <t>То же</t>
-        </is>
-      </c>
+          <t>content/nedeli-3-4_12.10-25.10/03-sr-14.10-mem-roditelskiy-chat/</t>
+        </is>
+      </c>
+      <c r="N33" s="5" t="inlineStr"/>
       <c r="O33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
@@ -2739,22 +2739,22 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>9. Неделя 2 — спикеры</t>
+          <t>10. Недели 3–4</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Чт 08.10 · Спикеры трека TEAM</t>
+          <t>Чт 15.10 · 5 фраз, которые удерживают после пробного</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Пост + карусель</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Спикеры</t>
+          <t>Польза</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -2788,19 +2788,15 @@
       </c>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>Ждём цифры опроса</t>
+          <t>Готов</t>
         </is>
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/4-cht-08.10-team.md · Figma</t>
-        </is>
-      </c>
-      <c r="N34" s="5" t="inlineStr">
-        <is>
-          <t>То же</t>
-        </is>
-      </c>
+          <t>content/nedeli-3-4_12.10-25.10/04-cht-15.10-5-fraz-posle-probnogo/</t>
+        </is>
+      </c>
+      <c r="N34" s="5" t="inlineStr"/>
       <c r="O34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
@@ -2809,22 +2805,22 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>9. Неделя 2 — спикеры</t>
+          <t>10. Недели 3–4</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Пт 09.10 · Спикеры треков GROWTH + FUTURE</t>
+          <t>Пт 16.10 · Мем «Нет / Да» + рилс «Полный зал»</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Пост + карусель</t>
+          <t>Мем + рилс</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Спикеры</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -2858,17 +2854,17 @@
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>Ждём цифры опроса</t>
+          <t>Готов</t>
         </is>
       </c>
       <c r="M35" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/5-pt-09.10-growth-future.md · Figma</t>
+          <t>content/nedeli-3-4_12.10-25.10/05-pt-16.10-mem-net-da/</t>
         </is>
       </c>
       <c r="N35" s="5" t="inlineStr">
         <is>
-          <t>То же</t>
+          <t>Рилс — под трендовый звук</t>
         </is>
       </c>
       <c r="O35" s="5" t="inlineStr"/>
@@ -2879,22 +2875,22 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>9. Неделя 2 — спикеры</t>
+          <t>10. Недели 3–4</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Сб 10.10 · «Все спикеры РЕШЕНО» — закрепить</t>
+          <t>Сб 17.10 · Как выглядит день на РЕШЕНО</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Пост + карусель</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Спикеры</t>
+          <t>Форум</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -2928,19 +2924,15 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Ждём цифры опроса</t>
+          <t>Готов</t>
         </is>
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/6-sb-10.10-vse-spikery.md · Figma</t>
-        </is>
-      </c>
-      <c r="N36" s="5" t="inlineStr">
-        <is>
-          <t>Открепить манифест, закрепить этот пост</t>
-        </is>
-      </c>
+          <t>content/nedeli-3-4_12.10-25.10/06-sb-17.10-den-na-reshno/</t>
+        </is>
+      </c>
+      <c r="N36" s="5" t="inlineStr"/>
       <c r="O36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
@@ -2949,22 +2941,22 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>9. Неделя 2 — спикеры</t>
+          <t>10. Недели 3–4</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Вс 11.10 · Опрос «Чей разбор ждёте больше всего?»</t>
+          <t>Вс 18.10 · Какой ты зубр сегодня?</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Опрос + сторис</t>
+          <t>Картинка</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Спикеры</t>
+          <t>Вовлечение</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -2998,12 +2990,12 @@
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>Ждём цифры опроса</t>
+          <t>Готов</t>
         </is>
       </c>
       <c r="M37" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/7-vs-11.10-opros.md · Figma</t>
+          <t>content/nedeli-3-4_12.10-25.10/07-vs-18.10-kakoy-ty-zubr/</t>
         </is>
       </c>
       <c r="N37" s="5" t="inlineStr"/>
@@ -3015,27 +3007,27 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>9. Неделя 2 — спикеры</t>
+          <t>10. Недели 3–4</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Каждый день · Сторис-отсчёт «До форума N дней» + сторис каждого спикера</t>
+          <t>Пн 19.10 · 6 цифр каждый понедельник</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Сторис</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Отсчёт</t>
+          <t>Польза</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Нужно</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -3069,23 +3061,1045 @@
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
+          <t>content/nedeli-3-4_12.10-25.10/08-pn-19.10-6-cifr-ponedelnika/</t>
+        </is>
+      </c>
+      <c r="N38" s="5" t="inlineStr"/>
+      <c r="O38" s="5" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>10. Недели 3–4</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Вт 20.10 · Мем «Ожидание / реальность: второй филиал»</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Мем</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Мем</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K39" s="4">
+        <f>IF(COUNTIF(F39:J39,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F39:J39,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Готов</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>content/nedeli-3-4_12.10-25.10/09-vt-20.10-mem-ozhidanie-realnost/</t>
+        </is>
+      </c>
+      <c r="N39" s="5" t="inlineStr"/>
+      <c r="O39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>10. Недели 3–4</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Ср 21.10 · 5 вопросов тренеру на собеседовании</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Карусель</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Польза</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K40" s="4">
+        <f>IF(COUNTIF(F40:J40,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F40:J40,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>Готов</t>
+        </is>
+      </c>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>content/nedeli-3-4_12.10-25.10/10-sr-21.10-sobesedovanie-trenera/</t>
+        </is>
+      </c>
+      <c r="N40" s="5" t="inlineStr"/>
+      <c r="O40" s="5" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>10. Недели 3–4</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Чт 22.10 · Мем «Уровни владельца» + рилс «Hot Seat»</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Мем + рилс</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Мем</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K41" s="4">
+        <f>IF(COUNTIF(F41:J41,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F41:J41,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Готов</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>content/nedeli-3-4_12.10-25.10/11-cht-22.10-mem-urovni/</t>
+        </is>
+      </c>
+      <c r="N41" s="5" t="inlineStr">
+        <is>
+          <t>Рилс — под трендовый звук</t>
+        </is>
+      </c>
+      <c r="O41" s="5" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>10. Недели 3–4</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Пт 23.10 · Business Live: подайте бизнес на разбор</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Карусель</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Форум</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K42" s="4">
+        <f>IF(COUNTIF(F42:J42,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F42:J42,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>Готов</t>
+        </is>
+      </c>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>content/nedeli-3-4_12.10-25.10/12-pt-23.10-business-live/</t>
+        </is>
+      </c>
+      <c r="N42" s="5" t="inlineStr">
+        <is>
+          <t>Ссылка на форму заявки</t>
+        </is>
+      </c>
+      <c r="O42" s="5" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>10. Недели 3–4</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Сб 24.10 · Вы покупаете не билет</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Карусель</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Продажа</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K43" s="4">
+        <f>IF(COUNTIF(F43:J43,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F43:J43,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>Готов</t>
+        </is>
+      </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>content/nedeli-3-4_12.10-25.10/13-sb-24.10-ne-bilet/</t>
+        </is>
+      </c>
+      <c r="N43" s="5" t="inlineStr">
+        <is>
+          <t>Проверить стартовую цену для первых 50</t>
+        </is>
+      </c>
+      <c r="O43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>10. Недели 3–4</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Вс 25.10 · Объясните, что вы владелец спортшколы…</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Картинка</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Вовлечение</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K44" s="4">
+        <f>IF(COUNTIF(F44:J44,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F44:J44,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>Готов</t>
+        </is>
+      </c>
+      <c r="M44" s="5" t="inlineStr">
+        <is>
+          <t>content/nedeli-3-4_12.10-25.10/14-vs-25.10-objasni/</t>
+        </is>
+      </c>
+      <c r="N44" s="5" t="inlineStr"/>
+      <c r="O44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>10. Недели 3–4</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Каждый день · Сторис-отсчёт 32 → 19 дней</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Сторис</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Отсчёт</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K45" s="4">
+        <f>IF(COUNTIF(F45:J45,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F45:J45,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>Готов</t>
+        </is>
+      </c>
+      <c r="M45" s="5" t="inlineStr">
+        <is>
+          <t>content/nedeli-3-4_12.10-25.10/storis-otschet/</t>
+        </is>
+      </c>
+      <c r="N45" s="5" t="inlineStr"/>
+      <c r="O45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Пн 05.10 · Тизер «На этой неделе раскрываем всех спикеров»</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Пост + сторис</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K46" s="4">
+        <f>IF(COUNTIF(F46:J46,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F46:J46,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L46" s="4" t="inlineStr">
+        <is>
+          <t>Готов</t>
+        </is>
+      </c>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/1-pn-05.10-tizer.md · Figma: «Неделя 2 — спикеры»</t>
+        </is>
+      </c>
+      <c r="N46" s="5" t="inlineStr"/>
+      <c r="O46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Вт 06.10 · Спикеры трека MONEY</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Пост + карусель</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K47" s="4">
+        <f>IF(COUNTIF(F47:J47,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F47:J47,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/2-vt-06.10-money.md · Figma</t>
+        </is>
+      </c>
+      <c r="N47" s="5" t="inlineStr">
+        <is>
+          <t>Нужны имена, должности, темы, фото, ники; пригласить спикеров соавторами</t>
+        </is>
+      </c>
+      <c r="O47" s="5" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Ср 07.10 · Спикеры трека CLIENT</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Пост + карусель</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K48" s="4">
+        <f>IF(COUNTIF(F48:J48,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F48:J48,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L48" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/3-sr-07.10-client.md · Figma</t>
+        </is>
+      </c>
+      <c r="N48" s="5" t="inlineStr">
+        <is>
+          <t>То же</t>
+        </is>
+      </c>
+      <c r="O48" s="5" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Чт 08.10 · Спикеры трека TEAM</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Пост + карусель</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K49" s="4">
+        <f>IF(COUNTIF(F49:J49,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F49:J49,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/4-cht-08.10-team.md · Figma</t>
+        </is>
+      </c>
+      <c r="N49" s="5" t="inlineStr">
+        <is>
+          <t>То же</t>
+        </is>
+      </c>
+      <c r="O49" s="5" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Пт 09.10 · Спикеры треков GROWTH + FUTURE</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Пост + карусель</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K50" s="4">
+        <f>IF(COUNTIF(F50:J50,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F50:J50,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L50" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M50" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/5-pt-09.10-growth-future.md · Figma</t>
+        </is>
+      </c>
+      <c r="N50" s="5" t="inlineStr">
+        <is>
+          <t>То же</t>
+        </is>
+      </c>
+      <c r="O50" s="5" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Сб 10.10 · «Все спикеры РЕШЕНО» — закрепить</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Пост + карусель</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K51" s="4">
+        <f>IF(COUNTIF(F51:J51,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F51:J51,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/6-sb-10.10-vse-spikery.md · Figma</t>
+        </is>
+      </c>
+      <c r="N51" s="5" t="inlineStr">
+        <is>
+          <t>Открепить манифест, закрепить этот пост</t>
+        </is>
+      </c>
+      <c r="O51" s="5" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Вс 11.10 · Опрос «Чей разбор ждёте больше всего?»</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Опрос + сторис</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K52" s="4">
+        <f>IF(COUNTIF(F52:J52,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F52:J52,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L52" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M52" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/7-vs-11.10-opros.md · Figma</t>
+        </is>
+      </c>
+      <c r="N52" s="5" t="inlineStr"/>
+      <c r="O52" s="5" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Каждый день · Сторис-отсчёт «До форума N дней» + сторис каждого спикера</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Сторис</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Отсчёт</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K53" s="4">
+        <f>IF(COUNTIF(F53:J53,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F53:J53,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>Готов</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
           <t>content/week-02_05.10-11.10/instagram/README.md · Figma</t>
         </is>
       </c>
-      <c r="N38" s="5" t="inlineStr">
+      <c r="N53" s="5" t="inlineStr">
         <is>
           <t>Вт 38, Ср 37, Чт 36, Пт 35, Сб 34, Вс 33</t>
         </is>
       </c>
-      <c r="O38" s="5" t="inlineStr"/>
+      <c r="O53" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:O38"/>
+  <autoFilter ref="A3:O53"/>
   <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F4:J88">
+  <conditionalFormatting sqref="F4:J103">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Выложено"</formula>
     </cfRule>
@@ -3096,26 +4110,26 @@
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K4:K88">
+  <conditionalFormatting sqref="K4:K103">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
       <formula>"Готово"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L88">
+  <conditionalFormatting sqref="L4:L103">
     <cfRule type="cellIs" priority="5" operator="notEqual" dxfId="3">
       <formula>"Готов"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:E38">
+  <conditionalFormatting sqref="A4:E53">
     <cfRule type="expression" priority="6" dxfId="4">
       <formula>$K4="Готово"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F4:J88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F4:J103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Нужно,Выложено,—"</formula1>
     </dataValidation>
-    <dataValidation sqref="L4:L88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L4:L103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Готов,Нужно снять,Нужно сделать,Ждём цифры опроса"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3180,11 +4194,11 @@
         </is>
       </c>
       <c r="B3" s="9">
-        <f>COUNTIF(План!F4:F88,"Нужно")+COUNTIF(План!F4:F88,"Выложено")</f>
+        <f>COUNTIF(План!F4:F103,"Нужно")+COUNTIF(План!F4:F103,"Выложено")</f>
         <v/>
       </c>
       <c r="C3" s="9">
-        <f>COUNTIF(План!F4:F88,"Выложено")</f>
+        <f>COUNTIF(План!F4:F103,"Выложено")</f>
         <v/>
       </c>
       <c r="D3" s="9">
@@ -3203,11 +4217,11 @@
         </is>
       </c>
       <c r="B4" s="9">
-        <f>COUNTIF(План!G4:G88,"Нужно")+COUNTIF(План!G4:G88,"Выложено")</f>
+        <f>COUNTIF(План!G4:G103,"Нужно")+COUNTIF(План!G4:G103,"Выложено")</f>
         <v/>
       </c>
       <c r="C4" s="9">
-        <f>COUNTIF(План!G4:G88,"Выложено")</f>
+        <f>COUNTIF(План!G4:G103,"Выложено")</f>
         <v/>
       </c>
       <c r="D4" s="9">
@@ -3226,11 +4240,11 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <f>COUNTIF(План!H4:H88,"Нужно")+COUNTIF(План!H4:H88,"Выложено")</f>
+        <f>COUNTIF(План!H4:H103,"Нужно")+COUNTIF(План!H4:H103,"Выложено")</f>
         <v/>
       </c>
       <c r="C5" s="9">
-        <f>COUNTIF(План!H4:H88,"Выложено")</f>
+        <f>COUNTIF(План!H4:H103,"Выложено")</f>
         <v/>
       </c>
       <c r="D5" s="9">
@@ -3249,11 +4263,11 @@
         </is>
       </c>
       <c r="B6" s="9">
-        <f>COUNTIF(План!I4:I88,"Нужно")+COUNTIF(План!I4:I88,"Выложено")</f>
+        <f>COUNTIF(План!I4:I103,"Нужно")+COUNTIF(План!I4:I103,"Выложено")</f>
         <v/>
       </c>
       <c r="C6" s="9">
-        <f>COUNTIF(План!I4:I88,"Выложено")</f>
+        <f>COUNTIF(План!I4:I103,"Выложено")</f>
         <v/>
       </c>
       <c r="D6" s="9">
@@ -3272,11 +4286,11 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>COUNTIF(План!J4:J88,"Нужно")+COUNTIF(План!J4:J88,"Выложено")</f>
+        <f>COUNTIF(План!J4:J103,"Нужно")+COUNTIF(План!J4:J103,"Выложено")</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>COUNTIF(План!J4:J88,"Выложено")</f>
+        <f>COUNTIF(План!J4:J103,"Выложено")</f>
         <v/>
       </c>
       <c r="D7" s="9">
@@ -3325,7 +4339,7 @@
         </is>
       </c>
       <c r="B10" s="13">
-        <f>COUNTA(План!C4:C88)</f>
+        <f>COUNTA(План!C4:C103)</f>
         <v/>
       </c>
       <c r="C10" s="13" t="n"/>
@@ -3339,7 +4353,7 @@
         </is>
       </c>
       <c r="B11" s="13">
-        <f>COUNTIF(План!K4:K88,"Готово")</f>
+        <f>COUNTIF(План!K4:K103,"Готово")</f>
         <v/>
       </c>
       <c r="C11" s="13" t="n"/>
@@ -3353,7 +4367,7 @@
         </is>
       </c>
       <c r="B12" s="13">
-        <f>COUNTIF(План!L4:L88,"&lt;&gt;Готов")-COUNTBLANK(План!L4:L88)</f>
+        <f>COUNTIF(План!L4:L103,"&lt;&gt;Готов")-COUNTBLANK(План!L4:L103)</f>
         <v/>
       </c>
       <c r="C12" s="13" t="n"/>

</xml_diff>

<commit_message>
Weeks 3–4: name contest with a ticket prize (rules, vote and winner stories); start price confirmed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015DfynR8ViCbDyQMuNVS5SH
</commit_message>
<xml_diff>
--- a/content/plan/kontent-plan-RESHENO.xlsx
+++ b/content/plan/kontent-plan-RESHENO.xlsx
@@ -2592,7 +2592,7 @@
       </c>
       <c r="N31" s="5" t="inlineStr">
         <is>
-          <t>Решить про подарок автору имени</t>
+          <t>Конкурс имени: приз — билет; итоги 18.10</t>
         </is>
       </c>
       <c r="O31" s="5" t="inlineStr"/>
@@ -3402,11 +3402,7 @@
           <t>content/nedeli-3-4_12.10-25.10/13-sb-24.10-ne-bilet/</t>
         </is>
       </c>
-      <c r="N43" s="5" t="inlineStr">
-        <is>
-          <t>Проверить стартовую цену для первых 50</t>
-        </is>
-      </c>
+      <c r="N43" s="5" t="inlineStr"/>
       <c r="O43" s="5" t="inlineStr"/>
     </row>
     <row r="44">

</xml_diff>

<commit_message>
Weeks 3–4 after review: formats carousel + zubr reel (12.10), branded checklist PDF, giveaway instead of name contest, B/W meme panel, wording fixes; schedules updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015DfynR8ViCbDyQMuNVS5SH
</commit_message>
<xml_diff>
--- a/content/plan/kontent-plan-RESHENO.xlsx
+++ b/content/plan/kontent-plan-RESHENO.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Как пользоваться" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'План'!$A$3:$O$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'План'!$A$3:$O$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O53"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2538,12 +2538,12 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Пн 12.10 · Знакомьтесь: это зубр + сбор имени</t>
+          <t>Пн 12.10 · Рилс с зубром + карусель «9 форматов форума»</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Карусель</t>
+          <t>Рилс + карусель</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -2587,14 +2587,10 @@
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/01-pn-12.10-znakomtes-zubr/</t>
-        </is>
-      </c>
-      <c r="N31" s="5" t="inlineStr">
-        <is>
-          <t>Конкурс имени: приз — билет; итоги 18.10</t>
-        </is>
-      </c>
+          <t>content/nedeli-3-4_12.10-25.10/01-pn-12.10-zubr-formaty/ · reels/reel5-zubr-znakomtes.mp4</t>
+        </is>
+      </c>
+      <c r="N31" s="5" t="inlineStr"/>
       <c r="O31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
@@ -2678,17 +2674,17 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Ср 14.10 · Мем «Родительский чат в 23:47»</t>
+          <t>Ср 14.10 · Розыгрыш билета (итоги 25.10)</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Мем</t>
+          <t>Карусель + сторис</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Мем</t>
+          <t>Розыгрыш</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2727,10 +2723,14 @@
       </c>
       <c r="M33" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/03-sr-14.10-mem-roditelskiy-chat/</t>
-        </is>
-      </c>
-      <c r="N33" s="5" t="inlineStr"/>
+          <t>content/nedeli-3-4_12.10-25.10/03-sr-14.10-rozygrysh-bileta/</t>
+        </is>
+      </c>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>Записать выбор победителя</t>
+        </is>
+      </c>
       <c r="O33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
@@ -2744,17 +2744,17 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Чт 15.10 · 5 фраз, которые удерживают после пробного</t>
+          <t>Ср 14.10 · Мем «Родительский чат в 23:47»</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Карусель</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Польза</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -2793,7 +2793,7 @@
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/04-cht-15.10-5-fraz-posle-probnogo/</t>
+          <t>content/nedeli-3-4_12.10-25.10/03-sr-14.10-mem-roditelskiy-chat/</t>
         </is>
       </c>
       <c r="N34" s="5" t="inlineStr"/>
@@ -2810,17 +2810,17 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Пт 16.10 · Мем «Нет / Да» + рилс «Полный зал»</t>
+          <t>Чт 15.10 · 5 фраз, которые удерживают после пробного</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Мем + рилс</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Мем</t>
+          <t>Польза</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -2859,14 +2859,10 @@
       </c>
       <c r="M35" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/05-pt-16.10-mem-net-da/</t>
-        </is>
-      </c>
-      <c r="N35" s="5" t="inlineStr">
-        <is>
-          <t>Рилс — под трендовый звук</t>
-        </is>
-      </c>
+          <t>content/nedeli-3-4_12.10-25.10/04-cht-15.10-5-fraz-posle-probnogo/</t>
+        </is>
+      </c>
+      <c r="N35" s="5" t="inlineStr"/>
       <c r="O35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
@@ -2880,17 +2876,17 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Сб 17.10 · Как выглядит день на РЕШЕНО</t>
+          <t>Пт 16.10 · Мем «Нет / Да» + рилс «Полный зал»</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Карусель</t>
+          <t>Мем + рилс</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Форум</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -2929,10 +2925,14 @@
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/06-sb-17.10-den-na-reshno/</t>
-        </is>
-      </c>
-      <c r="N36" s="5" t="inlineStr"/>
+          <t>content/nedeli-3-4_12.10-25.10/05-pt-16.10-mem-net-da/</t>
+        </is>
+      </c>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>Рилс — под трендовый звук</t>
+        </is>
+      </c>
       <c r="O36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
@@ -2946,17 +2946,17 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Вс 18.10 · Какой ты зубр сегодня?</t>
+          <t>Сб 17.10 · Как выглядит день на РЕШЕНО</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Картинка</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Вовлечение</t>
+          <t>Форум</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="M37" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/07-vs-18.10-kakoy-ty-zubr/</t>
+          <t>content/nedeli-3-4_12.10-25.10/06-sb-17.10-den-na-reshno/</t>
         </is>
       </c>
       <c r="N37" s="5" t="inlineStr"/>
@@ -3012,17 +3012,17 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Пн 19.10 · 6 цифр каждый понедельник</t>
+          <t>Вс 18.10 · Какой ты зубр сегодня?</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Карусель</t>
+          <t>Картинка</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Польза</t>
+          <t>Вовлечение</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -3061,7 +3061,7 @@
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/08-pn-19.10-6-cifr-ponedelnika/</t>
+          <t>content/nedeli-3-4_12.10-25.10/07-vs-18.10-kakoy-ty-zubr/</t>
         </is>
       </c>
       <c r="N38" s="5" t="inlineStr"/>
@@ -3078,17 +3078,17 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Вт 20.10 · Мем «Ожидание / реальность: второй филиал»</t>
+          <t>Пн 19.10 · 6 цифр каждый понедельник</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Мем</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Мем</t>
+          <t>Польза</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
@@ -3127,7 +3127,7 @@
       </c>
       <c r="M39" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/09-vt-20.10-mem-ozhidanie-realnost/</t>
+          <t>content/nedeli-3-4_12.10-25.10/08-pn-19.10-6-cifr-ponedelnika/</t>
         </is>
       </c>
       <c r="N39" s="5" t="inlineStr"/>
@@ -3144,17 +3144,17 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Ср 21.10 · 5 вопросов тренеру на собеседовании</t>
+          <t>Вт 20.10 · Мем «Ожидание / реальность: второй филиал»</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Карусель</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Польза</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
@@ -3193,7 +3193,7 @@
       </c>
       <c r="M40" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/10-sr-21.10-sobesedovanie-trenera/</t>
+          <t>content/nedeli-3-4_12.10-25.10/09-vt-20.10-mem-ozhidanie-realnost/</t>
         </is>
       </c>
       <c r="N40" s="5" t="inlineStr"/>
@@ -3210,17 +3210,17 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Чт 22.10 · Мем «Уровни владельца» + рилс «Hot Seat»</t>
+          <t>Ср 21.10 · 5 вопросов тренеру на собеседовании</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Мем + рилс</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Мем</t>
+          <t>Польза</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -3259,14 +3259,10 @@
       </c>
       <c r="M41" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/11-cht-22.10-mem-urovni/</t>
-        </is>
-      </c>
-      <c r="N41" s="5" t="inlineStr">
-        <is>
-          <t>Рилс — под трендовый звук</t>
-        </is>
-      </c>
+          <t>content/nedeli-3-4_12.10-25.10/10-sr-21.10-sobesedovanie-trenera/</t>
+        </is>
+      </c>
+      <c r="N41" s="5" t="inlineStr"/>
       <c r="O41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
@@ -3280,17 +3276,17 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Пт 23.10 · Business Live: подайте бизнес на разбор</t>
+          <t>Чт 22.10 · Мем «Уровни владельца» + рилс «Hot Seat»</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Карусель</t>
+          <t>Мем + рилс</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Форум</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
@@ -3329,12 +3325,12 @@
       </c>
       <c r="M42" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/12-pt-23.10-business-live/</t>
+          <t>content/nedeli-3-4_12.10-25.10/11-cht-22.10-mem-urovni/</t>
         </is>
       </c>
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>Ссылка ведёт на #business-live</t>
+          <t>Рилс — под трендовый звук</t>
         </is>
       </c>
       <c r="O42" s="5" t="inlineStr"/>
@@ -3350,7 +3346,7 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Сб 24.10 · Вы покупаете не билет</t>
+          <t>Пт 23.10 · Business Live: подайте бизнес на разбор</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
@@ -3360,7 +3356,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Продажа</t>
+          <t>Форум</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -3399,10 +3395,14 @@
       </c>
       <c r="M43" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/13-sb-24.10-ne-bilet/</t>
-        </is>
-      </c>
-      <c r="N43" s="5" t="inlineStr"/>
+          <t>content/nedeli-3-4_12.10-25.10/12-pt-23.10-business-live/</t>
+        </is>
+      </c>
+      <c r="N43" s="5" t="inlineStr">
+        <is>
+          <t>Ссылка ведёт на #business-live</t>
+        </is>
+      </c>
       <c r="O43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
@@ -3416,17 +3416,17 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Вс 25.10 · Объясните, что вы владелец спортшколы…</t>
+          <t>Сб 24.10 · Вы покупаете не билет</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Картинка</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Вовлечение</t>
+          <t>Продажа</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="M44" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/14-vs-25.10-objasni/</t>
+          <t>content/nedeli-3-4_12.10-25.10/13-sb-24.10-ne-bilet/</t>
         </is>
       </c>
       <c r="N44" s="5" t="inlineStr"/>
@@ -3482,22 +3482,22 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Каждый день · Сторис-отсчёт 32 → 19 дней</t>
+          <t>Вс 25.10 · Итоги розыгрыша билета</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Сторис</t>
+          <t>Картинка + сторис</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Отсчёт</t>
+          <t>Розыгрыш</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Нужно</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="M45" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/storis-otschet/</t>
+          <t>content/nedeli-3-4_12.10-25.10/14-vs-25.10-itogi-rozygrysha/</t>
         </is>
       </c>
       <c r="N45" s="5" t="inlineStr"/>
@@ -3543,27 +3543,27 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>9. Неделя 2 — спикеры</t>
+          <t>10. Недели 3–4</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Пн 05.10 · Тизер «На этой неделе раскрываем всех спикеров»</t>
+          <t>Каждый день · Сторис-отсчёт 32 → 19 дней</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Пост + сторис</t>
+          <t>Сторис</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Спикеры</t>
+          <t>Отсчёт</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Нужно</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="M46" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/1-pn-05.10-tizer.md · Figma: «Неделя 2 — спикеры»</t>
+          <t>content/nedeli-3-4_12.10-25.10/storis-otschet/</t>
         </is>
       </c>
       <c r="N46" s="5" t="inlineStr"/>
@@ -3614,12 +3614,12 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Вт 06.10 · Спикеры трека MONEY</t>
+          <t>Пн 05.10 · Тизер «На этой неделе раскрываем всех спикеров»</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Пост + карусель</t>
+          <t>Пост + сторис</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -3658,19 +3658,15 @@
       </c>
       <c r="L47" s="4" t="inlineStr">
         <is>
-          <t>Ждём цифры опроса</t>
+          <t>Готов</t>
         </is>
       </c>
       <c r="M47" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/2-vt-06.10-money.md · Figma</t>
-        </is>
-      </c>
-      <c r="N47" s="5" t="inlineStr">
-        <is>
-          <t>Нужны имена, должности, темы, фото, ники; пригласить спикеров соавторами</t>
-        </is>
-      </c>
+          <t>content/week-02_05.10-11.10/telegram/1-pn-05.10-tizer.md · Figma: «Неделя 2 — спикеры»</t>
+        </is>
+      </c>
+      <c r="N47" s="5" t="inlineStr"/>
       <c r="O47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
@@ -3684,7 +3680,7 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Ср 07.10 · Спикеры трека CLIENT</t>
+          <t>Вт 06.10 · Спикеры трека MONEY</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -3733,12 +3729,12 @@
       </c>
       <c r="M48" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/3-sr-07.10-client.md · Figma</t>
+          <t>content/week-02_05.10-11.10/telegram/2-vt-06.10-money.md · Figma</t>
         </is>
       </c>
       <c r="N48" s="5" t="inlineStr">
         <is>
-          <t>То же</t>
+          <t>Нужны имена, должности, темы, фото, ники; пригласить спикеров соавторами</t>
         </is>
       </c>
       <c r="O48" s="5" t="inlineStr"/>
@@ -3754,7 +3750,7 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Чт 08.10 · Спикеры трека TEAM</t>
+          <t>Ср 07.10 · Спикеры трека CLIENT</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
@@ -3803,7 +3799,7 @@
       </c>
       <c r="M49" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/4-cht-08.10-team.md · Figma</t>
+          <t>content/week-02_05.10-11.10/telegram/3-sr-07.10-client.md · Figma</t>
         </is>
       </c>
       <c r="N49" s="5" t="inlineStr">
@@ -3824,7 +3820,7 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Пт 09.10 · Спикеры треков GROWTH + FUTURE</t>
+          <t>Чт 08.10 · Спикеры трека TEAM</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
@@ -3873,7 +3869,7 @@
       </c>
       <c r="M50" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/5-pt-09.10-growth-future.md · Figma</t>
+          <t>content/week-02_05.10-11.10/telegram/4-cht-08.10-team.md · Figma</t>
         </is>
       </c>
       <c r="N50" s="5" t="inlineStr">
@@ -3894,7 +3890,7 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Сб 10.10 · «Все спикеры РЕШЕНО» — закрепить</t>
+          <t>Пт 09.10 · Спикеры треков GROWTH + FUTURE</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
@@ -3943,12 +3939,12 @@
       </c>
       <c r="M51" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/6-sb-10.10-vse-spikery.md · Figma</t>
+          <t>content/week-02_05.10-11.10/telegram/5-pt-09.10-growth-future.md · Figma</t>
         </is>
       </c>
       <c r="N51" s="5" t="inlineStr">
         <is>
-          <t>Открепить манифест, закрепить этот пост</t>
+          <t>То же</t>
         </is>
       </c>
       <c r="O51" s="5" t="inlineStr"/>
@@ -3964,12 +3960,12 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Вс 11.10 · Опрос «Чей разбор ждёте больше всего?»</t>
+          <t>Сб 10.10 · «Все спикеры РЕШЕНО» — закрепить</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Опрос + сторис</t>
+          <t>Пост + карусель</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -4013,10 +4009,14 @@
       </c>
       <c r="M52" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/7-vs-11.10-opros.md · Figma</t>
-        </is>
-      </c>
-      <c r="N52" s="5" t="inlineStr"/>
+          <t>content/week-02_05.10-11.10/telegram/6-sb-10.10-vse-spikery.md · Figma</t>
+        </is>
+      </c>
+      <c r="N52" s="5" t="inlineStr">
+        <is>
+          <t>Открепить манифест, закрепить этот пост</t>
+        </is>
+      </c>
       <c r="O52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
@@ -4030,22 +4030,22 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Каждый день · Сторис-отсчёт «До форума N дней» + сторис каждого спикера</t>
+          <t>Вс 11.10 · Опрос «Чей разбор ждёте больше всего?»</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Сторис</t>
+          <t>Опрос + сторис</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>Отсчёт</t>
+          <t>Спикеры</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Нужно</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -4074,28 +4074,94 @@
       </c>
       <c r="L53" s="4" t="inlineStr">
         <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/7-vs-11.10-opros.md · Figma</t>
+        </is>
+      </c>
+      <c r="N53" s="5" t="inlineStr"/>
+      <c r="O53" s="5" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>Каждый день · Сторис-отсчёт «До форума N дней» + сторис каждого спикера</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Сторис</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Отсчёт</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K54" s="4">
+        <f>IF(COUNTIF(F54:J54,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F54:J54,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L54" s="4" t="inlineStr">
+        <is>
           <t>Готов</t>
         </is>
       </c>
-      <c r="M53" s="5" t="inlineStr">
+      <c r="M54" s="5" t="inlineStr">
         <is>
           <t>content/week-02_05.10-11.10/instagram/README.md · Figma</t>
         </is>
       </c>
-      <c r="N53" s="5" t="inlineStr">
+      <c r="N54" s="5" t="inlineStr">
         <is>
           <t>Вт 38, Ср 37, Чт 36, Пт 35, Сб 34, Вс 33</t>
         </is>
       </c>
-      <c r="O53" s="5" t="inlineStr"/>
+      <c r="O54" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:O53"/>
+  <autoFilter ref="A3:O54"/>
   <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F4:J103">
+  <conditionalFormatting sqref="F4:J104">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Выложено"</formula>
     </cfRule>
@@ -4106,26 +4172,26 @@
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K4:K103">
+  <conditionalFormatting sqref="K4:K104">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
       <formula>"Готово"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L103">
+  <conditionalFormatting sqref="L4:L104">
     <cfRule type="cellIs" priority="5" operator="notEqual" dxfId="3">
       <formula>"Готов"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:E53">
+  <conditionalFormatting sqref="A4:E54">
     <cfRule type="expression" priority="6" dxfId="4">
       <formula>$K4="Готово"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F4:J103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F4:J104" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Нужно,Выложено,—"</formula1>
     </dataValidation>
-    <dataValidation sqref="L4:L103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L4:L104" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Готов,Нужно снять,Нужно сделать,Ждём цифры опроса"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4190,11 +4256,11 @@
         </is>
       </c>
       <c r="B3" s="9">
-        <f>COUNTIF(План!F4:F103,"Нужно")+COUNTIF(План!F4:F103,"Выложено")</f>
+        <f>COUNTIF(План!F4:F104,"Нужно")+COUNTIF(План!F4:F104,"Выложено")</f>
         <v/>
       </c>
       <c r="C3" s="9">
-        <f>COUNTIF(План!F4:F103,"Выложено")</f>
+        <f>COUNTIF(План!F4:F104,"Выложено")</f>
         <v/>
       </c>
       <c r="D3" s="9">
@@ -4213,11 +4279,11 @@
         </is>
       </c>
       <c r="B4" s="9">
-        <f>COUNTIF(План!G4:G103,"Нужно")+COUNTIF(План!G4:G103,"Выложено")</f>
+        <f>COUNTIF(План!G4:G104,"Нужно")+COUNTIF(План!G4:G104,"Выложено")</f>
         <v/>
       </c>
       <c r="C4" s="9">
-        <f>COUNTIF(План!G4:G103,"Выложено")</f>
+        <f>COUNTIF(План!G4:G104,"Выложено")</f>
         <v/>
       </c>
       <c r="D4" s="9">
@@ -4236,11 +4302,11 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <f>COUNTIF(План!H4:H103,"Нужно")+COUNTIF(План!H4:H103,"Выложено")</f>
+        <f>COUNTIF(План!H4:H104,"Нужно")+COUNTIF(План!H4:H104,"Выложено")</f>
         <v/>
       </c>
       <c r="C5" s="9">
-        <f>COUNTIF(План!H4:H103,"Выложено")</f>
+        <f>COUNTIF(План!H4:H104,"Выложено")</f>
         <v/>
       </c>
       <c r="D5" s="9">
@@ -4259,11 +4325,11 @@
         </is>
       </c>
       <c r="B6" s="9">
-        <f>COUNTIF(План!I4:I103,"Нужно")+COUNTIF(План!I4:I103,"Выложено")</f>
+        <f>COUNTIF(План!I4:I104,"Нужно")+COUNTIF(План!I4:I104,"Выложено")</f>
         <v/>
       </c>
       <c r="C6" s="9">
-        <f>COUNTIF(План!I4:I103,"Выложено")</f>
+        <f>COUNTIF(План!I4:I104,"Выложено")</f>
         <v/>
       </c>
       <c r="D6" s="9">
@@ -4282,11 +4348,11 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>COUNTIF(План!J4:J103,"Нужно")+COUNTIF(План!J4:J103,"Выложено")</f>
+        <f>COUNTIF(План!J4:J104,"Нужно")+COUNTIF(План!J4:J104,"Выложено")</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>COUNTIF(План!J4:J103,"Выложено")</f>
+        <f>COUNTIF(План!J4:J104,"Выложено")</f>
         <v/>
       </c>
       <c r="D7" s="9">
@@ -4335,7 +4401,7 @@
         </is>
       </c>
       <c r="B10" s="13">
-        <f>COUNTA(План!C4:C103)</f>
+        <f>COUNTA(План!C4:C104)</f>
         <v/>
       </c>
       <c r="C10" s="13" t="n"/>
@@ -4349,7 +4415,7 @@
         </is>
       </c>
       <c r="B11" s="13">
-        <f>COUNTIF(План!K4:K103,"Готово")</f>
+        <f>COUNTIF(План!K4:K104,"Готово")</f>
         <v/>
       </c>
       <c r="C11" s="13" t="n"/>
@@ -4363,7 +4429,7 @@
         </is>
       </c>
       <c r="B12" s="13">
-        <f>COUNTIF(План!L4:L103,"&lt;&gt;Готов")-COUNTBLANK(План!L4:L103)</f>
+        <f>COUNTIF(План!L4:L104,"&lt;&gt;Готов")-COUNTBLANK(План!L4:L104)</f>
         <v/>
       </c>
       <c r="C12" s="13" t="n"/>

</xml_diff>

<commit_message>
Week 27.10–02.11: texts, README, plan rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015DfynR8ViCbDyQMuNVS5SH
</commit_message>
<xml_diff>
--- a/content/plan/kontent-plan-RESHENO.xlsx
+++ b/content/plan/kontent-plan-RESHENO.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Как пользоваться" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'План'!$A$3:$O$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'План'!$A$3:$O$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2533,22 +2533,22 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>10. Недели 3–4</t>
+          <t>11. Неделя 27.10–02.11</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Пн 12.10 · Рилс с зубром + карусель «9 форматов форума»</t>
+          <t>Вт 27.10 · Зубр: «Вот такой вот спортбизнес, собачка»</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Рилс + карусель</t>
+          <t>Картинка</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Знакомство</t>
+          <t>Зубр</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -2582,15 +2582,19 @@
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>Готов</t>
+          <t>Нужно сделать</t>
         </is>
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/01-pn-12.10-zubr-formaty/ · reels/reel5-zubr-znakomtes.mp4</t>
-        </is>
-      </c>
-      <c r="N31" s="5" t="inlineStr"/>
+          <t>content/nedelya-5_27.10-02.11/01-zubr-sportbiznes/</t>
+        </is>
+      </c>
+      <c r="N31" s="5" t="inlineStr">
+        <is>
+          <t>Сгенерировать зубра в спортзале (промпт в tekst.md)</t>
+        </is>
+      </c>
       <c r="O31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
@@ -2599,22 +2603,22 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>10. Недели 3–4</t>
+          <t>11. Неделя 27.10–02.11</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Вт 13.10 · Сколько стоит потерянный клиент + чек-лист</t>
+          <t>Чт 29.10 · Схема зала «Места разбирают» + тарифы</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Карусель</t>
+          <t>Картинка</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Польза</t>
+          <t>Продажа</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -2653,12 +2657,12 @@
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/02-vt-13.10-poteryannyy-klient/</t>
+          <t>content/nedelya-5_27.10-02.11/02-skhema-zala/</t>
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>Сразу после поста — чек-лист в Telegram</t>
+          <t>Подставить ссылки [ЧАТ] [ВК]</t>
         </is>
       </c>
       <c r="O32" s="5" t="inlineStr"/>
@@ -2669,22 +2673,22 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>10. Недели 3–4</t>
+          <t>11. Неделя 27.10–02.11</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Ср 14.10 · Розыгрыш билета (итоги 25.10)</t>
+          <t>Сб 31.10 · Все спикеры в одном посте</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Карусель + сторис</t>
+          <t>Картинка</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Розыгрыш</t>
+          <t>Спикеры</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2718,17 +2722,17 @@
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>Готов</t>
+          <t>Ждём цифры опроса</t>
         </is>
       </c>
       <c r="M33" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/03-sr-14.10-rozygrysh-bileta/</t>
+          <t>content/nedelya-5_27.10-02.11/03-spikery-vmeste/</t>
         </is>
       </c>
       <c r="N33" s="5" t="inlineStr">
         <is>
-          <t>Записать выбор победителя</t>
+          <t>Кто есть кто на фото + данные 4 спикеров</t>
         </is>
       </c>
       <c r="O33" s="5" t="inlineStr"/>
@@ -2739,27 +2743,27 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>10. Недели 3–4</t>
+          <t>11. Неделя 27.10–02.11</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Ср 14.10 · Мем «Родительский чат в 23:47»</t>
+          <t>Пн 02.11 · Рилс «До форума 11 дней»</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Мем</t>
+          <t>Рилс</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Мем</t>
+          <t>Отсчёт</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Нужно</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -2793,10 +2797,14 @@
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/03-sr-14.10-mem-roditelskiy-chat/</t>
-        </is>
-      </c>
-      <c r="N34" s="5" t="inlineStr"/>
+          <t>reels/bez-muzyki/reel6-otschet-11-dney-bez-zvuka.mp4</t>
+        </is>
+      </c>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t>Трендовый трек в приложении</t>
+        </is>
+      </c>
       <c r="O34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
@@ -2810,17 +2818,17 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Чт 15.10 · 5 фраз, которые удерживают после пробного</t>
+          <t>Пн 12.10 · Рилс с зубром + карусель «9 форматов форума»</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Карусель</t>
+          <t>Рилс + карусель</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Польза</t>
+          <t>Знакомство</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -2859,7 +2867,7 @@
       </c>
       <c r="M35" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/04-cht-15.10-5-fraz-posle-probnogo/</t>
+          <t>content/nedeli-3-4_12.10-25.10/01-pn-12.10-zubr-formaty/ · reels/reel5-zubr-znakomtes.mp4</t>
         </is>
       </c>
       <c r="N35" s="5" t="inlineStr"/>
@@ -2876,17 +2884,17 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Пт 16.10 · Мем «Нет / Да» + рилс «Полный зал»</t>
+          <t>Вт 13.10 · Сколько стоит потерянный клиент + чек-лист</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Мем + рилс</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Мем</t>
+          <t>Польза</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -2925,12 +2933,12 @@
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/05-pt-16.10-mem-net-da/</t>
+          <t>content/nedeli-3-4_12.10-25.10/02-vt-13.10-poteryannyy-klient/</t>
         </is>
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>Рилс — под трендовый звук</t>
+          <t>Сразу после поста — чек-лист в Telegram</t>
         </is>
       </c>
       <c r="O36" s="5" t="inlineStr"/>
@@ -2946,17 +2954,17 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Сб 17.10 · Как выглядит день на РЕШЕНО</t>
+          <t>Ср 14.10 · Розыгрыш билета (итоги 25.10)</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Карусель</t>
+          <t>Карусель + сторис</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Форум</t>
+          <t>Розыгрыш</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -2995,10 +3003,14 @@
       </c>
       <c r="M37" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/06-sb-17.10-den-na-reshno/</t>
-        </is>
-      </c>
-      <c r="N37" s="5" t="inlineStr"/>
+          <t>content/nedeli-3-4_12.10-25.10/03-sr-14.10-rozygrysh-bileta/</t>
+        </is>
+      </c>
+      <c r="N37" s="5" t="inlineStr">
+        <is>
+          <t>Записать выбор победителя</t>
+        </is>
+      </c>
       <c r="O37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
@@ -3012,17 +3024,17 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Вс 18.10 · Какой ты зубр сегодня?</t>
+          <t>Ср 14.10 · Мем «Родительский чат в 23:47»</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Картинка</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Вовлечение</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -3061,7 +3073,7 @@
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/07-vs-18.10-kakoy-ty-zubr/</t>
+          <t>content/nedeli-3-4_12.10-25.10/03-sr-14.10-mem-roditelskiy-chat/</t>
         </is>
       </c>
       <c r="N38" s="5" t="inlineStr"/>
@@ -3078,7 +3090,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Пн 19.10 · 6 цифр каждый понедельник</t>
+          <t>Чт 15.10 · 5 фраз, которые удерживают после пробного</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -3127,7 +3139,7 @@
       </c>
       <c r="M39" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/08-pn-19.10-6-cifr-ponedelnika/</t>
+          <t>content/nedeli-3-4_12.10-25.10/04-cht-15.10-5-fraz-posle-probnogo/</t>
         </is>
       </c>
       <c r="N39" s="5" t="inlineStr"/>
@@ -3144,12 +3156,12 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Вт 20.10 · Мем «Ожидание / реальность: второй филиал»</t>
+          <t>Пт 16.10 · Мем «Нет / Да» + рилс «Полный зал»</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Мем</t>
+          <t>Мем + рилс</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -3193,10 +3205,14 @@
       </c>
       <c r="M40" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/09-vt-20.10-mem-ozhidanie-realnost/</t>
-        </is>
-      </c>
-      <c r="N40" s="5" t="inlineStr"/>
+          <t>content/nedeli-3-4_12.10-25.10/05-pt-16.10-mem-net-da/</t>
+        </is>
+      </c>
+      <c r="N40" s="5" t="inlineStr">
+        <is>
+          <t>Рилс — под трендовый звук</t>
+        </is>
+      </c>
       <c r="O40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
@@ -3210,7 +3226,7 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Ср 21.10 · 5 вопросов тренеру на собеседовании</t>
+          <t>Сб 17.10 · Как выглядит день на РЕШЕНО</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
@@ -3220,7 +3236,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Польза</t>
+          <t>Форум</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -3259,7 +3275,7 @@
       </c>
       <c r="M41" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/10-sr-21.10-sobesedovanie-trenera/</t>
+          <t>content/nedeli-3-4_12.10-25.10/06-sb-17.10-den-na-reshno/</t>
         </is>
       </c>
       <c r="N41" s="5" t="inlineStr"/>
@@ -3276,17 +3292,17 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Чт 22.10 · Мем «Уровни владельца» + рилс «Hot Seat»</t>
+          <t>Вс 18.10 · Какой ты зубр сегодня?</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Мем + рилс</t>
+          <t>Картинка</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Мем</t>
+          <t>Вовлечение</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
@@ -3325,14 +3341,10 @@
       </c>
       <c r="M42" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/11-cht-22.10-mem-urovni/</t>
-        </is>
-      </c>
-      <c r="N42" s="5" t="inlineStr">
-        <is>
-          <t>Рилс — под трендовый звук</t>
-        </is>
-      </c>
+          <t>content/nedeli-3-4_12.10-25.10/07-vs-18.10-kakoy-ty-zubr/</t>
+        </is>
+      </c>
+      <c r="N42" s="5" t="inlineStr"/>
       <c r="O42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
@@ -3346,7 +3358,7 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Пт 23.10 · Business Live: подайте бизнес на разбор</t>
+          <t>Пн 19.10 · 6 цифр каждый понедельник</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
@@ -3356,7 +3368,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Форум</t>
+          <t>Польза</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -3395,14 +3407,10 @@
       </c>
       <c r="M43" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/12-pt-23.10-business-live/</t>
-        </is>
-      </c>
-      <c r="N43" s="5" t="inlineStr">
-        <is>
-          <t>Ссылка ведёт на #business-live</t>
-        </is>
-      </c>
+          <t>content/nedeli-3-4_12.10-25.10/08-pn-19.10-6-cifr-ponedelnika/</t>
+        </is>
+      </c>
+      <c r="N43" s="5" t="inlineStr"/>
       <c r="O43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
@@ -3416,17 +3424,17 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Сб 24.10 · Вы покупаете не билет</t>
+          <t>Вт 20.10 · Мем «Ожидание / реальность: второй филиал»</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Карусель</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Продажа</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
@@ -3465,7 +3473,7 @@
       </c>
       <c r="M44" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/13-sb-24.10-ne-bilet/</t>
+          <t>content/nedeli-3-4_12.10-25.10/09-vt-20.10-mem-ozhidanie-realnost/</t>
         </is>
       </c>
       <c r="N44" s="5" t="inlineStr"/>
@@ -3482,17 +3490,17 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Вс 25.10 · Итоги розыгрыша билета</t>
+          <t>Ср 21.10 · 5 вопросов тренеру на собеседовании</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Картинка + сторис</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Розыгрыш</t>
+          <t>Польза</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -3531,7 +3539,7 @@
       </c>
       <c r="M45" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/14-vs-25.10-itogi-rozygrysha/</t>
+          <t>content/nedeli-3-4_12.10-25.10/10-sr-21.10-sobesedovanie-trenera/</t>
         </is>
       </c>
       <c r="N45" s="5" t="inlineStr"/>
@@ -3548,22 +3556,22 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Каждый день · Сторис-отсчёт 32 → 19 дней</t>
+          <t>Чт 22.10 · Мем «Уровни владельца» + рилс «Hot Seat»</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Сторис</t>
+          <t>Мем + рилс</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Отсчёт</t>
+          <t>Мем</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Нужно</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -3597,10 +3605,14 @@
       </c>
       <c r="M46" s="5" t="inlineStr">
         <is>
-          <t>content/nedeli-3-4_12.10-25.10/storis-otschet/</t>
-        </is>
-      </c>
-      <c r="N46" s="5" t="inlineStr"/>
+          <t>content/nedeli-3-4_12.10-25.10/11-cht-22.10-mem-urovni/</t>
+        </is>
+      </c>
+      <c r="N46" s="5" t="inlineStr">
+        <is>
+          <t>Рилс — под трендовый звук</t>
+        </is>
+      </c>
       <c r="O46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
@@ -3609,22 +3621,22 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>9. Неделя 2 — спикеры</t>
+          <t>10. Недели 3–4</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Пн 05.10 · Тизер «На этой неделе раскрываем всех спикеров»</t>
+          <t>Пт 23.10 · Business Live: подайте бизнес на разбор</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Пост + сторис</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Спикеры</t>
+          <t>Форум</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -3663,10 +3675,14 @@
       </c>
       <c r="M47" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/1-pn-05.10-tizer.md · Figma: «Неделя 2 — спикеры»</t>
-        </is>
-      </c>
-      <c r="N47" s="5" t="inlineStr"/>
+          <t>content/nedeli-3-4_12.10-25.10/12-pt-23.10-business-live/</t>
+        </is>
+      </c>
+      <c r="N47" s="5" t="inlineStr">
+        <is>
+          <t>Ссылка ведёт на #business-live</t>
+        </is>
+      </c>
       <c r="O47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
@@ -3675,22 +3691,22 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>9. Неделя 2 — спикеры</t>
+          <t>10. Недели 3–4</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Вт 06.10 · Спикеры трека MONEY</t>
+          <t>Сб 24.10 · Вы покупаете не билет</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Пост + карусель</t>
+          <t>Карусель</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Спикеры</t>
+          <t>Продажа</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
@@ -3724,19 +3740,15 @@
       </c>
       <c r="L48" s="4" t="inlineStr">
         <is>
-          <t>Ждём цифры опроса</t>
+          <t>Готов</t>
         </is>
       </c>
       <c r="M48" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/2-vt-06.10-money.md · Figma</t>
-        </is>
-      </c>
-      <c r="N48" s="5" t="inlineStr">
-        <is>
-          <t>Нужны имена, должности, темы, фото, ники; пригласить спикеров соавторами</t>
-        </is>
-      </c>
+          <t>content/nedeli-3-4_12.10-25.10/13-sb-24.10-ne-bilet/</t>
+        </is>
+      </c>
+      <c r="N48" s="5" t="inlineStr"/>
       <c r="O48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
@@ -3745,22 +3757,22 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>9. Неделя 2 — спикеры</t>
+          <t>10. Недели 3–4</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Ср 07.10 · Спикеры трека CLIENT</t>
+          <t>Вс 25.10 · Итоги розыгрыша билета</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Пост + карусель</t>
+          <t>Картинка + сторис</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Спикеры</t>
+          <t>Розыгрыш</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
@@ -3794,19 +3806,15 @@
       </c>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>Ждём цифры опроса</t>
+          <t>Готов</t>
         </is>
       </c>
       <c r="M49" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/3-sr-07.10-client.md · Figma</t>
-        </is>
-      </c>
-      <c r="N49" s="5" t="inlineStr">
-        <is>
-          <t>То же</t>
-        </is>
-      </c>
+          <t>content/nedeli-3-4_12.10-25.10/14-vs-25.10-itogi-rozygrysha/</t>
+        </is>
+      </c>
+      <c r="N49" s="5" t="inlineStr"/>
       <c r="O49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
@@ -3815,27 +3823,27 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>9. Неделя 2 — спикеры</t>
+          <t>10. Недели 3–4</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Чт 08.10 · Спикеры трека TEAM</t>
+          <t>Каждый день · Сторис-отсчёт 32 → 19 дней</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Пост + карусель</t>
+          <t>Сторис</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>Спикеры</t>
+          <t>Отсчёт</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Нужно</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -3864,19 +3872,15 @@
       </c>
       <c r="L50" s="4" t="inlineStr">
         <is>
-          <t>Ждём цифры опроса</t>
+          <t>Готов</t>
         </is>
       </c>
       <c r="M50" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/4-cht-08.10-team.md · Figma</t>
-        </is>
-      </c>
-      <c r="N50" s="5" t="inlineStr">
-        <is>
-          <t>То же</t>
-        </is>
-      </c>
+          <t>content/nedeli-3-4_12.10-25.10/storis-otschet/</t>
+        </is>
+      </c>
+      <c r="N50" s="5" t="inlineStr"/>
       <c r="O50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
@@ -3890,12 +3894,12 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Пт 09.10 · Спикеры треков GROWTH + FUTURE</t>
+          <t>Пн 05.10 · Тизер «На этой неделе раскрываем всех спикеров»</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Пост + карусель</t>
+          <t>Пост + сторис</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -3934,19 +3938,15 @@
       </c>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>Ждём цифры опроса</t>
+          <t>Готов</t>
         </is>
       </c>
       <c r="M51" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/5-pt-09.10-growth-future.md · Figma</t>
-        </is>
-      </c>
-      <c r="N51" s="5" t="inlineStr">
-        <is>
-          <t>То же</t>
-        </is>
-      </c>
+          <t>content/week-02_05.10-11.10/telegram/1-pn-05.10-tizer.md · Figma: «Неделя 2 — спикеры»</t>
+        </is>
+      </c>
+      <c r="N51" s="5" t="inlineStr"/>
       <c r="O51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Сб 10.10 · «Все спикеры РЕШЕНО» — закрепить</t>
+          <t>Вт 06.10 · Спикеры трека MONEY</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
@@ -4009,12 +4009,12 @@
       </c>
       <c r="M52" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/6-sb-10.10-vse-spikery.md · Figma</t>
+          <t>content/week-02_05.10-11.10/telegram/2-vt-06.10-money.md · Figma</t>
         </is>
       </c>
       <c r="N52" s="5" t="inlineStr">
         <is>
-          <t>Открепить манифест, закрепить этот пост</t>
+          <t>Нужны имена, должности, темы, фото, ники; пригласить спикеров соавторами</t>
         </is>
       </c>
       <c r="O52" s="5" t="inlineStr"/>
@@ -4030,12 +4030,12 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Вс 11.10 · Опрос «Чей разбор ждёте больше всего?»</t>
+          <t>Ср 07.10 · Спикеры трека CLIENT</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Опрос + сторис</t>
+          <t>Пост + карусель</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -4079,10 +4079,14 @@
       </c>
       <c r="M53" s="5" t="inlineStr">
         <is>
-          <t>content/week-02_05.10-11.10/telegram/7-vs-11.10-opros.md · Figma</t>
-        </is>
-      </c>
-      <c r="N53" s="5" t="inlineStr"/>
+          <t>content/week-02_05.10-11.10/telegram/3-sr-07.10-client.md · Figma</t>
+        </is>
+      </c>
+      <c r="N53" s="5" t="inlineStr">
+        <is>
+          <t>То же</t>
+        </is>
+      </c>
       <c r="O53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
@@ -4096,22 +4100,22 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Каждый день · Сторис-отсчёт «До форума N дней» + сторис каждого спикера</t>
+          <t>Чт 08.10 · Спикеры трека TEAM</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Сторис</t>
+          <t>Пост + карусель</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>Отсчёт</t>
+          <t>Спикеры</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Нужно</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -4140,28 +4144,304 @@
       </c>
       <c r="L54" s="4" t="inlineStr">
         <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M54" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/4-cht-08.10-team.md · Figma</t>
+        </is>
+      </c>
+      <c r="N54" s="5" t="inlineStr">
+        <is>
+          <t>То же</t>
+        </is>
+      </c>
+      <c r="O54" s="5" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Пт 09.10 · Спикеры треков GROWTH + FUTURE</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Пост + карусель</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K55" s="4">
+        <f>IF(COUNTIF(F55:J55,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F55:J55,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M55" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/5-pt-09.10-growth-future.md · Figma</t>
+        </is>
+      </c>
+      <c r="N55" s="5" t="inlineStr">
+        <is>
+          <t>То же</t>
+        </is>
+      </c>
+      <c r="O55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>Сб 10.10 · «Все спикеры РЕШЕНО» — закрепить</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Пост + карусель</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K56" s="4">
+        <f>IF(COUNTIF(F56:J56,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F56:J56,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M56" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/6-sb-10.10-vse-spikery.md · Figma</t>
+        </is>
+      </c>
+      <c r="N56" s="5" t="inlineStr">
+        <is>
+          <t>Открепить манифест, закрепить этот пост</t>
+        </is>
+      </c>
+      <c r="O56" s="5" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Вс 11.10 · Опрос «Чей разбор ждёте больше всего?»</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Опрос + сторис</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Спикеры</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K57" s="4">
+        <f>IF(COUNTIF(F57:J57,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F57:J57,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>Ждём цифры опроса</t>
+        </is>
+      </c>
+      <c r="M57" s="5" t="inlineStr">
+        <is>
+          <t>content/week-02_05.10-11.10/telegram/7-vs-11.10-opros.md · Figma</t>
+        </is>
+      </c>
+      <c r="N57" s="5" t="inlineStr"/>
+      <c r="O57" s="5" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>9. Неделя 2 — спикеры</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>Каждый день · Сторис-отсчёт «До форума N дней» + сторис каждого спикера</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Сторис</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Отсчёт</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>Нужно</t>
+        </is>
+      </c>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K58" s="4">
+        <f>IF(COUNTIF(F58:J58,"Нужно")=0,"Готово","Осталось: "&amp;COUNTIF(F58:J58,"Нужно"))</f>
+        <v/>
+      </c>
+      <c r="L58" s="4" t="inlineStr">
+        <is>
           <t>Готов</t>
         </is>
       </c>
-      <c r="M54" s="5" t="inlineStr">
+      <c r="M58" s="5" t="inlineStr">
         <is>
           <t>content/week-02_05.10-11.10/instagram/README.md · Figma</t>
         </is>
       </c>
-      <c r="N54" s="5" t="inlineStr">
+      <c r="N58" s="5" t="inlineStr">
         <is>
           <t>Вт 38, Ср 37, Чт 36, Пт 35, Сб 34, Вс 33</t>
         </is>
       </c>
-      <c r="O54" s="5" t="inlineStr"/>
+      <c r="O58" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:O54"/>
+  <autoFilter ref="A3:O58"/>
   <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F4:J104">
+  <conditionalFormatting sqref="F4:J108">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Выложено"</formula>
     </cfRule>
@@ -4172,26 +4452,26 @@
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K4:K104">
+  <conditionalFormatting sqref="K4:K108">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
       <formula>"Готово"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L104">
+  <conditionalFormatting sqref="L4:L108">
     <cfRule type="cellIs" priority="5" operator="notEqual" dxfId="3">
       <formula>"Готов"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:E54">
+  <conditionalFormatting sqref="A4:E58">
     <cfRule type="expression" priority="6" dxfId="4">
       <formula>$K4="Готово"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F4:J104" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F4:J108" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Нужно,Выложено,—"</formula1>
     </dataValidation>
-    <dataValidation sqref="L4:L104" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L4:L108" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Готов,Нужно снять,Нужно сделать,Ждём цифры опроса"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4256,11 +4536,11 @@
         </is>
       </c>
       <c r="B3" s="9">
-        <f>COUNTIF(План!F4:F104,"Нужно")+COUNTIF(План!F4:F104,"Выложено")</f>
+        <f>COUNTIF(План!F4:F108,"Нужно")+COUNTIF(План!F4:F108,"Выложено")</f>
         <v/>
       </c>
       <c r="C3" s="9">
-        <f>COUNTIF(План!F4:F104,"Выложено")</f>
+        <f>COUNTIF(План!F4:F108,"Выложено")</f>
         <v/>
       </c>
       <c r="D3" s="9">
@@ -4279,11 +4559,11 @@
         </is>
       </c>
       <c r="B4" s="9">
-        <f>COUNTIF(План!G4:G104,"Нужно")+COUNTIF(План!G4:G104,"Выложено")</f>
+        <f>COUNTIF(План!G4:G108,"Нужно")+COUNTIF(План!G4:G108,"Выложено")</f>
         <v/>
       </c>
       <c r="C4" s="9">
-        <f>COUNTIF(План!G4:G104,"Выложено")</f>
+        <f>COUNTIF(План!G4:G108,"Выложено")</f>
         <v/>
       </c>
       <c r="D4" s="9">
@@ -4302,11 +4582,11 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <f>COUNTIF(План!H4:H104,"Нужно")+COUNTIF(План!H4:H104,"Выложено")</f>
+        <f>COUNTIF(План!H4:H108,"Нужно")+COUNTIF(План!H4:H108,"Выложено")</f>
         <v/>
       </c>
       <c r="C5" s="9">
-        <f>COUNTIF(План!H4:H104,"Выложено")</f>
+        <f>COUNTIF(План!H4:H108,"Выложено")</f>
         <v/>
       </c>
       <c r="D5" s="9">
@@ -4325,11 +4605,11 @@
         </is>
       </c>
       <c r="B6" s="9">
-        <f>COUNTIF(План!I4:I104,"Нужно")+COUNTIF(План!I4:I104,"Выложено")</f>
+        <f>COUNTIF(План!I4:I108,"Нужно")+COUNTIF(План!I4:I108,"Выложено")</f>
         <v/>
       </c>
       <c r="C6" s="9">
-        <f>COUNTIF(План!I4:I104,"Выложено")</f>
+        <f>COUNTIF(План!I4:I108,"Выложено")</f>
         <v/>
       </c>
       <c r="D6" s="9">
@@ -4348,11 +4628,11 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>COUNTIF(План!J4:J104,"Нужно")+COUNTIF(План!J4:J104,"Выложено")</f>
+        <f>COUNTIF(План!J4:J108,"Нужно")+COUNTIF(План!J4:J108,"Выложено")</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>COUNTIF(План!J4:J104,"Выложено")</f>
+        <f>COUNTIF(План!J4:J108,"Выложено")</f>
         <v/>
       </c>
       <c r="D7" s="9">
@@ -4401,7 +4681,7 @@
         </is>
       </c>
       <c r="B10" s="13">
-        <f>COUNTA(План!C4:C104)</f>
+        <f>COUNTA(План!C4:C108)</f>
         <v/>
       </c>
       <c r="C10" s="13" t="n"/>
@@ -4415,7 +4695,7 @@
         </is>
       </c>
       <c r="B11" s="13">
-        <f>COUNTIF(План!K4:K104,"Готово")</f>
+        <f>COUNTIF(План!K4:K108,"Готово")</f>
         <v/>
       </c>
       <c r="C11" s="13" t="n"/>
@@ -4429,7 +4709,7 @@
         </is>
       </c>
       <c r="B12" s="13">
-        <f>COUNTIF(План!L4:L104,"&lt;&gt;Готов")-COUNTBLANK(План!L4:L104)</f>
+        <f>COUNTIF(План!L4:L108,"&lt;&gt;Готов")-COUNTBLANK(План!L4:L108)</f>
         <v/>
       </c>
       <c r="C12" s="13" t="n"/>

</xml_diff>